<commit_message>
added more methods to API
</commit_message>
<xml_diff>
--- a/api/Quiniela.xlsx
+++ b/api/Quiniela.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\wamp64\www\quiniela2026\api\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C83685B-8322-43DE-B8AF-F1C656B68E46}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{01C1597B-A007-4C82-B640-9B23914412DD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -262,7 +262,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -284,6 +284,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -354,7 +360,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -409,22 +415,25 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="16" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -715,7 +724,7 @@
     <col min="5" max="5" width="7.5546875" style="1" customWidth="1"/>
     <col min="6" max="6" width="20.109375" style="1" customWidth="1"/>
     <col min="7" max="7" width="8" style="1" customWidth="1"/>
-    <col min="8" max="8" width="10.109375" style="25" customWidth="1"/>
+    <col min="8" max="8" width="10.109375" style="23" customWidth="1"/>
     <col min="9" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
@@ -726,22 +735,22 @@
       <c r="C1" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="D1" s="20" t="s">
+      <c r="D1" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="E1" s="21"/>
-      <c r="F1" s="20" t="s">
+      <c r="E1" s="25"/>
+      <c r="F1" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="21"/>
-      <c r="H1" s="22"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="20"/>
     </row>
     <row r="2" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B2" s="5">
         <v>1</v>
       </c>
       <c r="C2" s="7">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="D2" s="2" t="s">
         <v>33</v>
@@ -751,14 +760,14 @@
         <v>51</v>
       </c>
       <c r="G2" s="2"/>
-      <c r="H2" s="23"/>
+      <c r="H2" s="21"/>
     </row>
     <row r="3" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B3" s="6">
         <v>2</v>
       </c>
       <c r="C3" s="8">
-        <v>46183</v>
+        <v>46184</v>
       </c>
       <c r="D3" s="3" t="s">
         <v>39</v>
@@ -768,14 +777,14 @@
         <v>37</v>
       </c>
       <c r="G3" s="3"/>
-      <c r="H3" s="23"/>
+      <c r="H3" s="21"/>
     </row>
     <row r="4" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B4" s="5">
         <v>3</v>
       </c>
       <c r="C4" s="7">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>40</v>
@@ -785,14 +794,14 @@
         <v>29</v>
       </c>
       <c r="G4" s="2"/>
-      <c r="H4" s="23"/>
+      <c r="H4" s="21"/>
     </row>
     <row r="5" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B5" s="6">
         <v>4</v>
       </c>
       <c r="C5" s="8">
-        <v>46184</v>
+        <v>46185</v>
       </c>
       <c r="D5" s="3" t="s">
         <v>0</v>
@@ -802,14 +811,14 @@
         <v>1</v>
       </c>
       <c r="G5" s="3"/>
-      <c r="H5" s="23"/>
+      <c r="H5" s="21"/>
     </row>
     <row r="6" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B6" s="5">
         <v>5</v>
       </c>
       <c r="C6" s="7">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="D6" s="2" t="s">
         <v>2</v>
@@ -819,14 +828,14 @@
         <v>3</v>
       </c>
       <c r="G6" s="2"/>
-      <c r="H6" s="23"/>
+      <c r="H6" s="21"/>
     </row>
     <row r="7" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B7" s="6">
         <v>6</v>
       </c>
       <c r="C7" s="8">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>4</v>
@@ -836,14 +845,14 @@
         <v>5</v>
       </c>
       <c r="G7" s="3"/>
-      <c r="H7" s="23"/>
+      <c r="H7" s="21"/>
     </row>
     <row r="8" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B8" s="5">
         <v>7</v>
       </c>
       <c r="C8" s="7">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="D8" s="2" t="s">
         <v>41</v>
@@ -853,14 +862,14 @@
         <v>6</v>
       </c>
       <c r="G8" s="2"/>
-      <c r="H8" s="23"/>
+      <c r="H8" s="21"/>
     </row>
     <row r="9" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="6">
         <v>8</v>
       </c>
       <c r="C9" s="8">
-        <v>46185</v>
+        <v>46186</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>7</v>
@@ -870,14 +879,14 @@
         <v>48</v>
       </c>
       <c r="G9" s="3"/>
-      <c r="H9" s="23"/>
+      <c r="H9" s="21"/>
     </row>
     <row r="10" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="5">
         <v>9</v>
       </c>
       <c r="C10" s="7">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>9</v>
@@ -887,14 +896,14 @@
         <v>8</v>
       </c>
       <c r="G10" s="2"/>
-      <c r="H10" s="23"/>
+      <c r="H10" s="21"/>
     </row>
     <row r="11" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="6">
         <v>10</v>
       </c>
       <c r="C11" s="8">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>42</v>
@@ -904,14 +913,14 @@
         <v>32</v>
       </c>
       <c r="G11" s="3"/>
-      <c r="H11" s="23"/>
+      <c r="H11" s="21"/>
     </row>
     <row r="12" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B12" s="5">
         <v>11</v>
       </c>
       <c r="C12" s="7">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>11</v>
@@ -921,14 +930,14 @@
         <v>10</v>
       </c>
       <c r="G12" s="2"/>
-      <c r="H12" s="23"/>
+      <c r="H12" s="21"/>
     </row>
     <row r="13" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B13" s="6">
         <v>12</v>
       </c>
       <c r="C13" s="8">
-        <v>46186</v>
+        <v>46187</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>28</v>
@@ -938,14 +947,14 @@
         <v>49</v>
       </c>
       <c r="G13" s="3"/>
-      <c r="H13" s="23"/>
+      <c r="H13" s="21"/>
     </row>
     <row r="14" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B14" s="5">
         <v>13</v>
       </c>
       <c r="C14" s="7">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>13</v>
@@ -955,14 +964,14 @@
         <v>12</v>
       </c>
       <c r="G14" s="2"/>
-      <c r="H14" s="23"/>
+      <c r="H14" s="21"/>
     </row>
     <row r="15" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B15" s="6">
         <v>14</v>
       </c>
       <c r="C15" s="8">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="D15" s="3" t="s">
         <v>43</v>
@@ -972,14 +981,14 @@
         <v>14</v>
       </c>
       <c r="G15" s="3"/>
-      <c r="H15" s="23"/>
+      <c r="H15" s="21"/>
     </row>
     <row r="16" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B16" s="5">
         <v>15</v>
       </c>
       <c r="C16" s="7">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="D16" s="2" t="s">
         <v>44</v>
@@ -989,14 +998,14 @@
         <v>15</v>
       </c>
       <c r="G16" s="2"/>
-      <c r="H16" s="23"/>
+      <c r="H16" s="21"/>
     </row>
     <row r="17" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B17" s="6">
         <v>16</v>
       </c>
       <c r="C17" s="8">
-        <v>46187</v>
+        <v>46188</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>45</v>
@@ -1006,14 +1015,14 @@
         <v>16</v>
       </c>
       <c r="G17" s="3"/>
-      <c r="H17" s="23"/>
+      <c r="H17" s="21"/>
     </row>
     <row r="18" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B18" s="5">
         <v>17</v>
       </c>
       <c r="C18" s="7">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>17</v>
@@ -1023,14 +1032,14 @@
         <v>18</v>
       </c>
       <c r="G18" s="2"/>
-      <c r="H18" s="23"/>
+      <c r="H18" s="21"/>
     </row>
     <row r="19" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B19" s="6">
         <v>18</v>
       </c>
       <c r="C19" s="8">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="D19" s="3" t="s">
         <v>30</v>
@@ -1040,14 +1049,14 @@
         <v>19</v>
       </c>
       <c r="G19" s="3"/>
-      <c r="H19" s="23"/>
+      <c r="H19" s="21"/>
     </row>
     <row r="20" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B20" s="5">
         <v>19</v>
       </c>
       <c r="C20" s="7">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>21</v>
@@ -1057,14 +1066,14 @@
         <v>20</v>
       </c>
       <c r="G20" s="2"/>
-      <c r="H20" s="23"/>
+      <c r="H20" s="21"/>
     </row>
     <row r="21" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B21" s="6">
         <v>20</v>
       </c>
       <c r="C21" s="8">
-        <v>46188</v>
+        <v>46189</v>
       </c>
       <c r="D21" s="3" t="s">
         <v>22</v>
@@ -1074,14 +1083,14 @@
         <v>23</v>
       </c>
       <c r="G21" s="3"/>
-      <c r="H21" s="23"/>
+      <c r="H21" s="21"/>
     </row>
     <row r="22" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B22" s="5">
         <v>21</v>
       </c>
       <c r="C22" s="7">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>24</v>
@@ -1091,14 +1100,14 @@
         <v>38</v>
       </c>
       <c r="G22" s="2"/>
-      <c r="H22" s="23"/>
+      <c r="H22" s="21"/>
     </row>
     <row r="23" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B23" s="6">
         <v>22</v>
       </c>
       <c r="C23" s="8">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>26</v>
@@ -1108,14 +1117,14 @@
         <v>25</v>
       </c>
       <c r="G23" s="3"/>
-      <c r="H23" s="23"/>
+      <c r="H23" s="21"/>
     </row>
     <row r="24" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B24" s="5">
         <v>23</v>
       </c>
       <c r="C24" s="7">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>46</v>
@@ -1125,14 +1134,14 @@
         <v>50</v>
       </c>
       <c r="G24" s="2"/>
-      <c r="H24" s="23"/>
+      <c r="H24" s="21"/>
     </row>
     <row r="25" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B25" s="6">
         <v>24</v>
       </c>
       <c r="C25" s="8">
-        <v>46189</v>
+        <v>46190</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>47</v>
@@ -1142,14 +1151,14 @@
         <v>27</v>
       </c>
       <c r="G25" s="3"/>
-      <c r="H25" s="23"/>
+      <c r="H25" s="21"/>
     </row>
     <row r="26" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B26" s="5">
         <v>25</v>
       </c>
       <c r="C26" s="7">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="D26" s="2" t="s">
         <v>37</v>
@@ -1159,14 +1168,14 @@
         <v>51</v>
       </c>
       <c r="G26" s="2"/>
-      <c r="H26" s="23"/>
+      <c r="H26" s="21"/>
     </row>
     <row r="27" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B27" s="6">
         <v>26</v>
       </c>
       <c r="C27" s="8">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>3</v>
@@ -1176,14 +1185,14 @@
         <v>29</v>
       </c>
       <c r="G27" s="3"/>
-      <c r="H27" s="23"/>
+      <c r="H27" s="21"/>
     </row>
     <row r="28" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B28" s="5">
         <v>27</v>
       </c>
       <c r="C28" s="7">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="D28" s="2" t="s">
         <v>40</v>
@@ -1193,14 +1202,14 @@
         <v>2</v>
       </c>
       <c r="G28" s="2"/>
-      <c r="H28" s="23"/>
+      <c r="H28" s="21"/>
     </row>
     <row r="29" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B29" s="6">
         <v>28</v>
       </c>
       <c r="C29" s="8">
-        <v>46190</v>
+        <v>46191</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>33</v>
@@ -1210,14 +1219,14 @@
         <v>39</v>
       </c>
       <c r="G29" s="3"/>
-      <c r="H29" s="23"/>
+      <c r="H29" s="21"/>
     </row>
     <row r="30" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B30" s="5">
         <v>29</v>
       </c>
       <c r="C30" s="7">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="D30" s="2" t="s">
         <v>0</v>
@@ -1227,14 +1236,14 @@
         <v>7</v>
       </c>
       <c r="G30" s="2"/>
-      <c r="H30" s="23"/>
+      <c r="H30" s="21"/>
     </row>
     <row r="31" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B31" s="6">
         <v>30</v>
       </c>
       <c r="C31" s="8">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>6</v>
@@ -1244,14 +1253,14 @@
         <v>5</v>
       </c>
       <c r="G31" s="3"/>
-      <c r="H31" s="23"/>
+      <c r="H31" s="21"/>
     </row>
     <row r="32" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B32" s="5">
         <v>31</v>
       </c>
       <c r="C32" s="7">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="D32" s="2" t="s">
         <v>4</v>
@@ -1261,14 +1270,14 @@
         <v>41</v>
       </c>
       <c r="G32" s="2"/>
-      <c r="H32" s="23"/>
+      <c r="H32" s="21"/>
     </row>
     <row r="33" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B33" s="6">
         <v>32</v>
       </c>
       <c r="C33" s="8">
-        <v>46191</v>
+        <v>46192</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>48</v>
@@ -1278,14 +1287,14 @@
         <v>1</v>
       </c>
       <c r="G33" s="3"/>
-      <c r="H33" s="23"/>
+      <c r="H33" s="21"/>
     </row>
     <row r="34" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B34" s="5">
         <v>33</v>
       </c>
-      <c r="C34" s="7">
-        <v>46192</v>
+      <c r="C34" s="10">
+        <v>46193</v>
       </c>
       <c r="D34" s="2" t="s">
         <v>42</v>
@@ -1295,14 +1304,14 @@
         <v>28</v>
       </c>
       <c r="G34" s="2"/>
-      <c r="H34" s="23"/>
+      <c r="H34" s="21"/>
     </row>
     <row r="35" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B35" s="6">
         <v>34</v>
       </c>
-      <c r="C35" s="8">
-        <v>46192</v>
+      <c r="C35" s="13">
+        <v>46193</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>9</v>
@@ -1312,14 +1321,14 @@
         <v>11</v>
       </c>
       <c r="G35" s="3"/>
-      <c r="H35" s="23"/>
+      <c r="H35" s="21"/>
     </row>
     <row r="36" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B36" s="5">
         <v>35</v>
       </c>
-      <c r="C36" s="7">
-        <v>46192</v>
+      <c r="C36" s="16">
+        <v>46193</v>
       </c>
       <c r="D36" s="2" t="s">
         <v>10</v>
@@ -1329,14 +1338,14 @@
         <v>8</v>
       </c>
       <c r="G36" s="2"/>
-      <c r="H36" s="23"/>
+      <c r="H36" s="21"/>
     </row>
     <row r="37" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B37" s="6">
         <v>36</v>
       </c>
-      <c r="C37" s="8">
-        <v>46192</v>
+      <c r="C37" s="13">
+        <v>46193</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>49</v>
@@ -1346,7 +1355,7 @@
         <v>32</v>
       </c>
       <c r="G37" s="3"/>
-      <c r="H37" s="23"/>
+      <c r="H37" s="21"/>
     </row>
     <row r="38" spans="2:8" s="18" customFormat="1" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B38" s="19" t="s">
@@ -1355,22 +1364,22 @@
       <c r="C38" s="19" t="s">
         <v>34</v>
       </c>
-      <c r="D38" s="20" t="s">
+      <c r="D38" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="E38" s="21"/>
-      <c r="F38" s="20" t="s">
+      <c r="E38" s="25"/>
+      <c r="F38" s="24" t="s">
         <v>36</v>
       </c>
-      <c r="G38" s="21"/>
-      <c r="H38" s="22"/>
+      <c r="G38" s="25"/>
+      <c r="H38" s="20"/>
     </row>
     <row r="39" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B39" s="9">
         <v>37</v>
       </c>
-      <c r="C39" s="10">
-        <v>46193</v>
+      <c r="C39" s="16">
+        <v>46194</v>
       </c>
       <c r="D39" s="11" t="s">
         <v>13</v>
@@ -1380,14 +1389,14 @@
         <v>44</v>
       </c>
       <c r="G39" s="11"/>
-      <c r="H39" s="23"/>
+      <c r="H39" s="21"/>
     </row>
     <row r="40" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B40" s="12">
         <v>38</v>
       </c>
       <c r="C40" s="13">
-        <v>46193</v>
+        <v>46194</v>
       </c>
       <c r="D40" s="14" t="s">
         <v>43</v>
@@ -1397,14 +1406,14 @@
         <v>45</v>
       </c>
       <c r="G40" s="14"/>
-      <c r="H40" s="24"/>
+      <c r="H40" s="22"/>
     </row>
     <row r="41" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B41" s="15">
         <v>39</v>
       </c>
       <c r="C41" s="16">
-        <v>46193</v>
+        <v>46194</v>
       </c>
       <c r="D41" s="17" t="s">
         <v>15</v>
@@ -1414,14 +1423,14 @@
         <v>12</v>
       </c>
       <c r="G41" s="17"/>
-      <c r="H41" s="24"/>
+      <c r="H41" s="22"/>
     </row>
     <row r="42" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B42" s="12">
         <v>40</v>
       </c>
       <c r="C42" s="13">
-        <v>46193</v>
+        <v>46194</v>
       </c>
       <c r="D42" s="14" t="s">
         <v>16</v>
@@ -1431,14 +1440,14 @@
         <v>14</v>
       </c>
       <c r="G42" s="14"/>
-      <c r="H42" s="24"/>
+      <c r="H42" s="22"/>
     </row>
     <row r="43" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B43" s="15">
         <v>41</v>
       </c>
       <c r="C43" s="16">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="D43" s="17" t="s">
         <v>21</v>
@@ -1448,14 +1457,14 @@
         <v>22</v>
       </c>
       <c r="G43" s="17"/>
-      <c r="H43" s="24"/>
+      <c r="H43" s="22"/>
     </row>
     <row r="44" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B44" s="12">
         <v>42</v>
       </c>
       <c r="C44" s="13">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="D44" s="14" t="s">
         <v>17</v>
@@ -1465,14 +1474,14 @@
         <v>30</v>
       </c>
       <c r="G44" s="14"/>
-      <c r="H44" s="24"/>
+      <c r="H44" s="22"/>
     </row>
     <row r="45" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B45" s="15">
         <v>43</v>
       </c>
       <c r="C45" s="16">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="D45" s="17" t="s">
         <v>19</v>
@@ -1482,14 +1491,14 @@
         <v>18</v>
       </c>
       <c r="G45" s="17"/>
-      <c r="H45" s="24"/>
+      <c r="H45" s="22"/>
     </row>
     <row r="46" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B46" s="12">
         <v>44</v>
       </c>
       <c r="C46" s="13">
-        <v>46194</v>
+        <v>46195</v>
       </c>
       <c r="D46" s="14" t="s">
         <v>23</v>
@@ -1499,14 +1508,14 @@
         <v>20</v>
       </c>
       <c r="G46" s="14"/>
-      <c r="H46" s="24"/>
+      <c r="H46" s="22"/>
     </row>
     <row r="47" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B47" s="15">
         <v>45</v>
       </c>
       <c r="C47" s="16">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="D47" s="17" t="s">
         <v>24</v>
@@ -1516,14 +1525,14 @@
         <v>47</v>
       </c>
       <c r="G47" s="17"/>
-      <c r="H47" s="24"/>
+      <c r="H47" s="22"/>
     </row>
     <row r="48" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B48" s="12">
         <v>46</v>
       </c>
       <c r="C48" s="13">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="D48" s="14" t="s">
         <v>26</v>
@@ -1533,14 +1542,14 @@
         <v>46</v>
       </c>
       <c r="G48" s="14"/>
-      <c r="H48" s="24"/>
+      <c r="H48" s="22"/>
     </row>
     <row r="49" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B49" s="15">
         <v>47</v>
       </c>
       <c r="C49" s="16">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="D49" s="17" t="s">
         <v>50</v>
@@ -1550,14 +1559,14 @@
         <v>25</v>
       </c>
       <c r="G49" s="17"/>
-      <c r="H49" s="24"/>
+      <c r="H49" s="22"/>
     </row>
     <row r="50" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B50" s="12">
         <v>48</v>
       </c>
       <c r="C50" s="13">
-        <v>46195</v>
+        <v>46196</v>
       </c>
       <c r="D50" s="14" t="s">
         <v>27</v>
@@ -1567,14 +1576,14 @@
         <v>38</v>
       </c>
       <c r="G50" s="14"/>
-      <c r="H50" s="24"/>
+      <c r="H50" s="22"/>
     </row>
     <row r="51" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B51" s="15">
         <v>49</v>
       </c>
-      <c r="C51" s="16">
-        <v>46196</v>
+      <c r="C51" s="26">
+        <v>46197</v>
       </c>
       <c r="D51" s="17" t="s">
         <v>3</v>
@@ -1584,14 +1593,14 @@
         <v>40</v>
       </c>
       <c r="G51" s="17"/>
-      <c r="H51" s="24"/>
+      <c r="H51" s="22"/>
     </row>
     <row r="52" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B52" s="12">
         <v>50</v>
       </c>
       <c r="C52" s="13">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="D52" s="14" t="s">
         <v>29</v>
@@ -1601,14 +1610,14 @@
         <v>2</v>
       </c>
       <c r="G52" s="14"/>
-      <c r="H52" s="24"/>
+      <c r="H52" s="22"/>
     </row>
     <row r="53" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B53" s="15">
         <v>51</v>
       </c>
-      <c r="C53" s="16">
-        <v>46196</v>
+      <c r="C53" s="26">
+        <v>46197</v>
       </c>
       <c r="D53" s="17" t="s">
         <v>6</v>
@@ -1618,14 +1627,14 @@
         <v>4</v>
       </c>
       <c r="G53" s="17"/>
-      <c r="H53" s="24"/>
+      <c r="H53" s="22"/>
     </row>
     <row r="54" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B54" s="12">
         <v>52</v>
       </c>
       <c r="C54" s="13">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="D54" s="14" t="s">
         <v>5</v>
@@ -1635,14 +1644,14 @@
         <v>41</v>
       </c>
       <c r="G54" s="14"/>
-      <c r="H54" s="24"/>
+      <c r="H54" s="22"/>
     </row>
     <row r="55" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B55" s="15">
         <v>53</v>
       </c>
-      <c r="C55" s="16">
-        <v>46196</v>
+      <c r="C55" s="26">
+        <v>46197</v>
       </c>
       <c r="D55" s="17" t="s">
         <v>37</v>
@@ -1652,14 +1661,14 @@
         <v>33</v>
       </c>
       <c r="G55" s="17"/>
-      <c r="H55" s="24"/>
+      <c r="H55" s="22"/>
     </row>
     <row r="56" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B56" s="12">
         <v>54</v>
       </c>
       <c r="C56" s="13">
-        <v>46196</v>
+        <v>46197</v>
       </c>
       <c r="D56" s="14" t="s">
         <v>51</v>
@@ -1669,14 +1678,14 @@
         <v>39</v>
       </c>
       <c r="G56" s="14"/>
-      <c r="H56" s="24"/>
+      <c r="H56" s="22"/>
     </row>
     <row r="57" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B57" s="15">
         <v>55</v>
       </c>
       <c r="C57" s="16">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="D57" s="17" t="s">
         <v>8</v>
@@ -1686,14 +1695,14 @@
         <v>11</v>
       </c>
       <c r="G57" s="17"/>
-      <c r="H57" s="24"/>
+      <c r="H57" s="22"/>
     </row>
     <row r="58" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B58" s="12">
         <v>56</v>
       </c>
       <c r="C58" s="13">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="D58" s="14" t="s">
         <v>10</v>
@@ -1703,14 +1712,14 @@
         <v>9</v>
       </c>
       <c r="G58" s="14"/>
-      <c r="H58" s="24"/>
+      <c r="H58" s="22"/>
     </row>
     <row r="59" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B59" s="15">
         <v>57</v>
       </c>
       <c r="C59" s="16">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="D59" s="17" t="s">
         <v>32</v>
@@ -1720,14 +1729,14 @@
         <v>28</v>
       </c>
       <c r="G59" s="17"/>
-      <c r="H59" s="24"/>
+      <c r="H59" s="22"/>
     </row>
     <row r="60" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B60" s="12">
         <v>58</v>
       </c>
       <c r="C60" s="13">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="D60" s="14" t="s">
         <v>49</v>
@@ -1737,14 +1746,14 @@
         <v>42</v>
       </c>
       <c r="G60" s="14"/>
-      <c r="H60" s="24"/>
+      <c r="H60" s="22"/>
     </row>
     <row r="61" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B61" s="15">
         <v>59</v>
       </c>
       <c r="C61" s="16">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="D61" s="17" t="s">
         <v>48</v>
@@ -1754,14 +1763,14 @@
         <v>0</v>
       </c>
       <c r="G61" s="17"/>
-      <c r="H61" s="24"/>
+      <c r="H61" s="22"/>
     </row>
     <row r="62" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B62" s="12">
         <v>60</v>
       </c>
       <c r="C62" s="13">
-        <v>46197</v>
+        <v>46198</v>
       </c>
       <c r="D62" s="14" t="s">
         <v>1</v>
@@ -1771,14 +1780,14 @@
         <v>7</v>
       </c>
       <c r="G62" s="14"/>
-      <c r="H62" s="24"/>
+      <c r="H62" s="22"/>
     </row>
     <row r="63" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B63" s="15">
         <v>61</v>
       </c>
       <c r="C63" s="16">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="D63" s="17" t="s">
         <v>19</v>
@@ -1788,14 +1797,14 @@
         <v>17</v>
       </c>
       <c r="G63" s="17"/>
-      <c r="H63" s="24"/>
+      <c r="H63" s="22"/>
     </row>
     <row r="64" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B64" s="12">
         <v>62</v>
       </c>
       <c r="C64" s="13">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="D64" s="14" t="s">
         <v>18</v>
@@ -1805,14 +1814,14 @@
         <v>30</v>
       </c>
       <c r="G64" s="14"/>
-      <c r="H64" s="24"/>
+      <c r="H64" s="22"/>
     </row>
     <row r="65" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B65" s="15">
         <v>63</v>
       </c>
       <c r="C65" s="16">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="D65" s="17" t="s">
         <v>12</v>
@@ -1822,14 +1831,14 @@
         <v>44</v>
       </c>
       <c r="G65" s="17"/>
-      <c r="H65" s="24"/>
+      <c r="H65" s="22"/>
     </row>
     <row r="66" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B66" s="12">
         <v>64</v>
       </c>
       <c r="C66" s="13">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="D66" s="14" t="s">
         <v>15</v>
@@ -1839,14 +1848,14 @@
         <v>13</v>
       </c>
       <c r="G66" s="14"/>
-      <c r="H66" s="24"/>
+      <c r="H66" s="22"/>
     </row>
     <row r="67" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B67" s="15">
         <v>65</v>
       </c>
       <c r="C67" s="16">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="D67" s="17" t="s">
         <v>14</v>
@@ -1856,14 +1865,14 @@
         <v>45</v>
       </c>
       <c r="G67" s="17"/>
-      <c r="H67" s="24"/>
+      <c r="H67" s="22"/>
     </row>
     <row r="68" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B68" s="12">
         <v>66</v>
       </c>
       <c r="C68" s="13">
-        <v>46198</v>
+        <v>46199</v>
       </c>
       <c r="D68" s="14" t="s">
         <v>16</v>
@@ -1873,14 +1882,14 @@
         <v>43</v>
       </c>
       <c r="G68" s="14"/>
-      <c r="H68" s="24"/>
+      <c r="H68" s="22"/>
     </row>
     <row r="69" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B69" s="15">
         <v>67</v>
       </c>
       <c r="C69" s="16">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="D69" s="17" t="s">
         <v>50</v>
@@ -1890,14 +1899,14 @@
         <v>26</v>
       </c>
       <c r="G69" s="17"/>
-      <c r="H69" s="24"/>
+      <c r="H69" s="22"/>
     </row>
     <row r="70" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B70" s="12">
         <v>68</v>
       </c>
       <c r="C70" s="13">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="D70" s="14" t="s">
         <v>25</v>
@@ -1907,14 +1916,14 @@
         <v>46</v>
       </c>
       <c r="G70" s="14"/>
-      <c r="H70" s="24"/>
+      <c r="H70" s="22"/>
     </row>
     <row r="71" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B71" s="15">
         <v>69</v>
       </c>
       <c r="C71" s="16">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="D71" s="17" t="s">
         <v>27</v>
@@ -1924,14 +1933,14 @@
         <v>24</v>
       </c>
       <c r="G71" s="17"/>
-      <c r="H71" s="24"/>
+      <c r="H71" s="22"/>
     </row>
     <row r="72" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B72" s="12">
         <v>70</v>
       </c>
       <c r="C72" s="13">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="D72" s="14" t="s">
         <v>38</v>
@@ -1941,14 +1950,14 @@
         <v>47</v>
       </c>
       <c r="G72" s="14"/>
-      <c r="H72" s="24"/>
+      <c r="H72" s="22"/>
     </row>
     <row r="73" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B73" s="15">
         <v>71</v>
       </c>
       <c r="C73" s="16">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="D73" s="17" t="s">
         <v>20</v>
@@ -1958,14 +1967,14 @@
         <v>22</v>
       </c>
       <c r="G73" s="17"/>
-      <c r="H73" s="24"/>
+      <c r="H73" s="22"/>
     </row>
     <row r="74" spans="2:8" ht="19.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B74" s="12">
         <v>72</v>
       </c>
       <c r="C74" s="13">
-        <v>46199</v>
+        <v>46200</v>
       </c>
       <c r="D74" s="14" t="s">
         <v>23</v>
@@ -1975,7 +1984,7 @@
         <v>21</v>
       </c>
       <c r="G74" s="14"/>
-      <c r="H74" s="24"/>
+      <c r="H74" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>